<commit_message>
push local changes from Lenovo
</commit_message>
<xml_diff>
--- a/Dario Kulici LB2 BewertungsrasterV25_26.xlsx
+++ b/Dario Kulici LB2 BewertungsrasterV25_26.xlsx
@@ -295,15 +295,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -311,15 +311,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -574,7 +574,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.9140625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.73"/>
@@ -604,12 +604,12 @@
         <v>2</v>
       </c>
       <c r="H1" s="3" t="n">
-        <f aca="false">E1/(COUNTA(D4:D14,F4:F14,H4:H14))*5+1</f>
-        <v>3.72727272727273</v>
+        <f aca="false">E1/(COUNTA(D4:D12,F4:F12,H4:H12))*5+1</f>
+        <v>4.33333333333333</v>
       </c>
       <c r="I1" s="1" t="n">
         <f aca="false">ROUND(H1,1.1)</f>
-        <v>3.7</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>